<commit_message>
Se agraga el Proyecto
</commit_message>
<xml_diff>
--- a/Porticos 2D/P delta/comprobacion.xlsx
+++ b/Porticos 2D/P delta/comprobacion.xlsx
@@ -1,29 +1,62 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Poli\ELEMENTOS FINITOS\Elementos finitos_1\Porticos 2D\P delta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Poli\ELEMENTOS FINITOS\Elementos finitos_1\Porticos 2D\P delta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B038EA2-BA6F-402A-A165-18222E0D0C56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9293A53-CC0F-438E-A9C8-F68B216E62A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{FB349FF0-057F-40C8-8EC0-ED68B3DC8CB9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FB349FF0-057F-40C8-8EC0-ED68B3DC8CB9}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="Ac">Hoja1!$C$21</definedName>
+    <definedName name="D">Hoja1!$F$14</definedName>
     <definedName name="E">Hoja1!$C$17</definedName>
     <definedName name="EI">Hoja1!$C$20</definedName>
     <definedName name="G">Hoja1!$C$18</definedName>
     <definedName name="I">Hoja1!$C$19</definedName>
     <definedName name="L">Hoja1!$C$15</definedName>
-    <definedName name="landa">Hoja1!$C$23</definedName>
+    <definedName name="landa">Hoja1!$C$24</definedName>
+    <definedName name="mu">Hoja1!$F$13</definedName>
+    <definedName name="Omega">Hoja1!$F$12</definedName>
     <definedName name="P">Hoja1!$C$16</definedName>
+    <definedName name="solver_adj" localSheetId="0" hidden="1">Hoja1!$D$22</definedName>
+    <definedName name="solver_cvg" localSheetId="0" hidden="1">0.0001</definedName>
+    <definedName name="solver_drv" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="0" hidden="1">Hoja1!$E$31</definedName>
+    <definedName name="solver_mip" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
+    <definedName name="solver_mrt" localSheetId="0" hidden="1">0.075</definedName>
+    <definedName name="solver_msl" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_nod" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_num" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="0" hidden="1">Hoja1!$C$27</definedName>
+    <definedName name="solver_pre" localSheetId="0" hidden="1">0.000001</definedName>
+    <definedName name="solver_rbv" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rhs1" localSheetId="0" hidden="1">Hoja1!$F$31</definedName>
+    <definedName name="solver_rlx" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rsd" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_scl" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_sho" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_ssz" localSheetId="0" hidden="1">100</definedName>
+    <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_tol" localSheetId="0" hidden="1">0.01</definedName>
+    <definedName name="solver_typ" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
     <definedName name="X">Hoja1!$C$22</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -36,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Pdelta</t>
   </si>
@@ -93,14 +126,33 @@
   </si>
   <si>
     <t>I(m4)</t>
+  </si>
+  <si>
+    <t>P/(X*EI)</t>
+  </si>
+  <si>
+    <t>Version diego</t>
+  </si>
+  <si>
+    <t>vesion sap 2000</t>
+  </si>
+  <si>
+    <t>mu</t>
+  </si>
+  <si>
+    <t>Omega</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.000000000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0000000000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -174,17 +226,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -206,16 +273,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>140677</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>133607</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>503359</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>15643</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>373583</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>74042</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>736265</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>146578</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -239,8 +306,184 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4331677" y="4515107"/>
+          <a:off x="6687282" y="5884508"/>
           <a:ext cx="6328906" cy="1273935"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>232475</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>36634</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>735939</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>89176</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A09F0BC-1377-8DEB-5D88-9601802D12BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11750398" y="36634"/>
+          <a:ext cx="4313464" cy="5159407"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>721179</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>81643</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>730227</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>176714</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2E8D0BD-67A9-D394-C717-4BC787DE9519}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9701893" y="462643"/>
+          <a:ext cx="3819048" cy="1428571"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>761999</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>13607</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>637713</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>184869</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4B03624-0AE7-12A5-6DA4-38477C37C953}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9742713" y="1918607"/>
+          <a:ext cx="3685714" cy="1504762"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>511840</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>163287</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>520888</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>67858</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Imagen 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A9CC10A-992C-C24D-5134-749A17B17BC4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="12791763" y="3401787"/>
+          <a:ext cx="3819048" cy="1428571"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -549,21 +792,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2598A5FC-1B94-439C-BBBF-F7A8591BE350}">
-  <dimension ref="B1:G55"/>
+  <dimension ref="B1:M56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B1" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="6"/>
-    </row>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="13"/>
+    </row>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="1">
         <v>9361.1470000000008</v>
       </c>
@@ -571,7 +814,7 @@
         <v>19222.293399999999</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="1">
         <v>19222.293399999999</v>
       </c>
@@ -579,13 +822,13 @@
         <v>25513.8871</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="1">
         <v>0</v>
       </c>
       <c r="C4" s="1"/>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <f>+B2</f>
         <v>9361.1470000000008</v>
@@ -594,7 +837,7 @@
         <v>19222.293399999999</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <f>-B3</f>
         <v>-19222.293399999999</v>
@@ -603,21 +846,25 @@
         <v>51375.286599999999</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="6" t="s">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="6"/>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C8" s="13"/>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>9658.277</v>
       </c>
       <c r="C9" s="1">
         <v>19316.553</v>
       </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="E9">
+        <f>20*L^2/12</f>
+        <v>26.666666666666668</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <v>19316.553</v>
       </c>
@@ -625,27 +872,47 @@
         <v>25369.073</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12" s="1">
         <v>9658.277</v>
       </c>
       <c r="C12" s="1">
         <v>19316.553</v>
       </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12">
+        <f xml:space="preserve"> EI/(Ac*L^2)</f>
+        <v>2.5000000000000005E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13" s="1">
         <v>-19316.553</v>
       </c>
       <c r="C13" s="1">
         <v>51897.1391</v>
       </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13">
+        <f>SQRT(P/(EI*(1 + P/(Ac))))</f>
+        <v>0.13723615973940506</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F14">
+        <f>(2-2*COS(mu*L))*(1+Omega*mu^2*L^2)-mu*L*SIN((mu*L))</f>
+        <v>7.637733819082837E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
         <v>14</v>
       </c>
@@ -653,23 +920,33 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="1">
         <v>1000</v>
       </c>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E16" s="10"/>
+      <c r="F16" s="11">
+        <f xml:space="preserve"> (12*EI/L^3) * (mu*L)^3 * (1 - Omega*mu^2*L^2) * SIN(mu*L) / D</f>
+        <v>112337.33598918717</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="1">
         <v>24870062</v>
       </c>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E17" s="10"/>
+      <c r="F17" s="11">
+        <f>(6*EI/L^2)*(mu*L)^2*(1-COS(mu*L))/D</f>
+        <v>115332.88304423154</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>17</v>
       </c>
@@ -677,8 +954,13 @@
         <f>0.4*E</f>
         <v>9948024.8000000007</v>
       </c>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E18" s="10"/>
+      <c r="F18" s="12">
+        <f>(4*EI/L) * (mu*L*((1 + Omega*mu^2*L^2)*SIN(mu*L) - mu*L*COS(mu*L))) / (4*D)</f>
+        <v>51373.560253706484</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>18</v>
       </c>
@@ -687,7 +969,7 @@
         <v>2.1333333333333343E-3</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>2</v>
       </c>
@@ -695,8 +977,12 @@
         <f>+C19*C17</f>
         <v>53056.132266666689</v>
       </c>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="H20">
+        <f>+(1-P/Ac)^2*SQRT(P/((1-P/Ac)*EI)*L^2)^3*SIN(SQRT(P/((1-P/Ac)*EI)*L^2))/(2-2*COS(SQRT(P/((1-P/Ac)*EI)*L^2))-(1-P/Ac)*SQRT(P/((1-P/Ac)*EI)*L^2)*SIN(SQRT(P/((1-P/Ac)*EI)*L^2)))*EI/L^3</f>
+        <v>9361.0021942844396</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
         <v>3</v>
       </c>
@@ -704,245 +990,502 @@
         <f>0.4^2*G*5/6</f>
         <v>1326403.3066666669</v>
       </c>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E21">
+        <f>+G46</f>
+        <v>51372.767588837502</v>
+      </c>
+      <c r="H21">
+        <f>SQRT(P/(X*EI)*L^2)</f>
+        <v>0.54935865460584365</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C22" s="1">
-        <f>1-P/Ac</f>
+        <f>(1-P/Ac)</f>
         <v>0.99924608149348404</v>
       </c>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E22">
+        <f>+G45</f>
+        <v>-19222.0046215824</v>
+      </c>
+      <c r="L22">
+        <v>-9375.1402256090096</v>
+      </c>
+      <c r="M22">
+        <v>19236.143901481999</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23">
+        <f>P/(X*EI)</f>
+        <v>1.8862183211896411E-2</v>
+      </c>
+      <c r="E23">
+        <f>+G46</f>
+        <v>51372.767588837502</v>
+      </c>
+      <c r="J23">
+        <v>19236.1584039669</v>
+      </c>
+      <c r="K23">
+        <v>51372.324076173201</v>
+      </c>
+      <c r="L23">
+        <v>-19236.1584039669</v>
+      </c>
+      <c r="M23">
+        <v>25514.299600169099</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B24" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C23" s="1">
-        <f>SQRT(P*L^2/(X*EI))</f>
+      <c r="C24" s="7">
+        <f>SQRT(C23*L^2)</f>
         <v>0.54935865460584365</v>
       </c>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B24" s="1" t="s">
+      <c r="E24">
+        <f>+C42</f>
+        <v>9361.0023107912093</v>
+      </c>
+      <c r="J24">
+        <v>-9375.1402256090096</v>
+      </c>
+      <c r="K24">
+        <v>-19236.143901481999</v>
+      </c>
+      <c r="L24">
+        <v>9375.1402256090096</v>
+      </c>
+      <c r="M24">
+        <v>-19236.143901481999</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C24" s="1">
-        <f>2-2*COS(landa)-X*landa*SIN(landa)</f>
+      <c r="C25" s="1">
+        <f>(2-2*COS(landa)-X*landa*SIN(landa))</f>
         <v>7.6547912108466121E-3</v>
       </c>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C25" t="s">
+      <c r="J25">
+        <v>19236.1584039669</v>
+      </c>
+      <c r="L25">
+        <v>-19236.1584039669</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
         <v>13</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D26" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E26" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F25" s="4"/>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B26" s="2" t="s">
+      <c r="F26" s="4"/>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="3">
-        <f>+X^2*landa^3*SIN(landa)/C24*EI/L^3</f>
+      <c r="C27" s="3">
+        <f>+X^2*landa^3*SIN(landa)/C25*EI/L^3</f>
         <v>9361.0021942844396</v>
       </c>
-      <c r="D26">
+      <c r="D27">
         <f>+B2</f>
         <v>9361.1470000000008</v>
       </c>
-      <c r="E26" s="5">
-        <f>+D26/C26</f>
+      <c r="E27" s="5">
+        <f>+D27/C27</f>
         <v>1.0000154690398053</v>
       </c>
-      <c r="F26" s="5"/>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B27" s="2" t="s">
+      <c r="F27" s="5"/>
+      <c r="G27">
+        <f>(12*Ac*EI)/(L*(Ac*L^2 + 12*EI))</f>
+        <v>9658.2765048543733</v>
+      </c>
+      <c r="I27">
+        <v>9375.1402256090096</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B28" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C27" s="2">
-        <f>+X*landa^2*(1-COS(landa))/C24*EI/L^2</f>
+      <c r="C28" s="2">
+        <f>+X*landa^2*(1-COS(landa))/C25*EI/L^2</f>
         <v>19222.004388568879</v>
       </c>
-      <c r="D27">
+      <c r="D28">
         <f>+B3</f>
         <v>19222.293399999999</v>
       </c>
-      <c r="E27" s="5">
-        <f t="shared" ref="E27:E29" si="0">+D27/C27</f>
+      <c r="E28" s="5">
+        <f t="shared" ref="E28:E30" si="0">+D28/C28</f>
         <v>1.0000150354471509</v>
       </c>
-      <c r="F27" s="5"/>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B28" s="2" t="s">
+      <c r="F28" s="5"/>
+      <c r="G28">
+        <f>(6*Ac*EI)/(Ac*L^2 + 12*EI)</f>
+        <v>19316.553009708747</v>
+      </c>
+      <c r="I28">
+        <v>19236.143901481999</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B29" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C28" s="2">
-        <f>landa*(SIN(landa)-X*landa*COS(landa))/C24*EI/L</f>
+      <c r="C29" s="2">
+        <f>landa*(SIN(landa)-X*landa*COS(landa))/C25*EI/L</f>
         <v>51372.766962786583</v>
       </c>
-      <c r="D28">
+      <c r="D29">
         <f>+C6</f>
         <v>51375.286599999999</v>
       </c>
-      <c r="E28" s="4">
+      <c r="E29" s="4">
         <f t="shared" si="0"/>
         <v>1.0000490461651645</v>
       </c>
-      <c r="F28" s="4"/>
-    </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B29" s="2" t="s">
+      <c r="F29" s="4"/>
+      <c r="G29">
+        <f>(4*EI*(Ac*L^2 + 3*EI))/(L*(Ac*L^2 + 12*EI))</f>
+        <v>51897.139086084164</v>
+      </c>
+      <c r="I29">
+        <v>51372.324076173201</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C29" s="2">
-        <f>landa*(X*landa-SIN(landa))/C24*EI/L</f>
+      <c r="C30" s="8">
+        <f>landa*(X*landa-SIN(landa))/C25*EI/L</f>
         <v>25515.250591488886</v>
       </c>
-      <c r="D29">
+      <c r="D30">
         <f>+C3</f>
         <v>25513.8871</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E30" s="4">
         <f t="shared" si="0"/>
         <v>0.99994656170496943</v>
       </c>
-      <c r="F29" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30">
+        <f>-(2*EI*(- Ac*L^2 + 6*EI))/(L*(Ac*L^2 + 12*EI))</f>
+        <v>25369.072952750819</v>
+      </c>
+      <c r="I30">
+        <v>25514.299600169099</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E31" s="9">
+        <f>AVERAGE(E27:E30)</f>
+        <v>1.0000065280892725</v>
+      </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B33">
+      <c r="B33" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="1">
         <v>994802.48</v>
       </c>
-      <c r="C33">
-        <v>0</v>
-      </c>
-      <c r="D33">
-        <v>0</v>
-      </c>
-      <c r="E33">
+      <c r="C34" s="1">
+        <v>0</v>
+      </c>
+      <c r="D34" s="1">
+        <v>0</v>
+      </c>
+      <c r="E34" s="1">
         <v>-994802.48</v>
       </c>
-      <c r="F33">
-        <v>0</v>
-      </c>
-      <c r="G33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B34">
-        <v>0</v>
-      </c>
-      <c r="C34">
-        <v>9361.0021942846106</v>
-      </c>
-      <c r="D34">
-        <v>19222.004388569199</v>
-      </c>
-      <c r="E34">
-        <v>0</v>
-      </c>
-      <c r="F34">
-        <v>-9361.0021942846106</v>
-      </c>
-      <c r="G34">
-        <v>19222.004388569199</v>
+      <c r="F34" s="1">
+        <v>0</v>
+      </c>
+      <c r="G34" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B35">
-        <v>0</v>
-      </c>
-      <c r="C35">
-        <v>19222.004388569199</v>
-      </c>
-      <c r="D35">
-        <v>51372.7669627875</v>
-      </c>
-      <c r="E35">
-        <v>0</v>
-      </c>
-      <c r="F35">
-        <v>-19222.004388569199</v>
-      </c>
-      <c r="G35">
-        <v>25515.250591489301</v>
+      <c r="B35" s="1">
+        <v>0</v>
+      </c>
+      <c r="C35" s="7">
+        <f>+D27</f>
+        <v>9361.1470000000008</v>
+      </c>
+      <c r="D35" s="1">
+        <f>+D28</f>
+        <v>19222.293399999999</v>
+      </c>
+      <c r="E35" s="1">
+        <v>0</v>
+      </c>
+      <c r="F35" s="1">
+        <f>-D27</f>
+        <v>-9361.1470000000008</v>
+      </c>
+      <c r="G35" s="1">
+        <f>+D28</f>
+        <v>19222.293399999999</v>
       </c>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B36">
+      <c r="B36" s="1">
+        <v>0</v>
+      </c>
+      <c r="C36" s="1">
+        <f>+D28</f>
+        <v>19222.293399999999</v>
+      </c>
+      <c r="D36" s="1">
+        <f>+D29</f>
+        <v>51375.286599999999</v>
+      </c>
+      <c r="E36" s="1">
+        <v>0</v>
+      </c>
+      <c r="F36" s="1">
+        <f>-D28</f>
+        <v>-19222.293399999999</v>
+      </c>
+      <c r="G36" s="1">
+        <f>+D30</f>
+        <v>25513.8871</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="1">
         <v>-994802.48</v>
       </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
-      <c r="D36">
-        <v>0</v>
-      </c>
-      <c r="E36">
+      <c r="C37" s="1">
+        <v>0</v>
+      </c>
+      <c r="D37" s="1">
+        <v>0</v>
+      </c>
+      <c r="E37" s="1">
         <v>994802.48</v>
       </c>
-      <c r="F36">
-        <v>0</v>
-      </c>
-      <c r="G36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B37">
-        <v>0</v>
-      </c>
-      <c r="C37">
-        <v>-9361.0021942846106</v>
-      </c>
-      <c r="D37">
-        <v>-19222.004388569199</v>
-      </c>
-      <c r="E37">
-        <v>0</v>
-      </c>
-      <c r="F37">
-        <v>9361.0021942846106</v>
-      </c>
-      <c r="G37">
-        <v>-19222.004388569199</v>
+      <c r="F37" s="1">
+        <v>0</v>
+      </c>
+      <c r="G37" s="1">
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B38">
-        <v>0</v>
-      </c>
-      <c r="C38">
-        <v>19222.004388569199</v>
-      </c>
-      <c r="D38">
-        <v>25515.250591489301</v>
-      </c>
-      <c r="E38">
-        <v>0</v>
-      </c>
-      <c r="F38">
-        <v>-19222.004388569199</v>
-      </c>
-      <c r="G38">
-        <v>51372.7669627875</v>
-      </c>
-    </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B55" s="7"/>
+      <c r="B38" s="1">
+        <v>0</v>
+      </c>
+      <c r="C38" s="1">
+        <f>-D27</f>
+        <v>-9361.1470000000008</v>
+      </c>
+      <c r="D38" s="1">
+        <f>-D28</f>
+        <v>-19222.293399999999</v>
+      </c>
+      <c r="E38" s="1">
+        <v>0</v>
+      </c>
+      <c r="F38" s="1">
+        <f>+D28</f>
+        <v>19222.293399999999</v>
+      </c>
+      <c r="G38" s="1">
+        <f>-D28</f>
+        <v>-19222.293399999999</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="1">
+        <v>0</v>
+      </c>
+      <c r="C39" s="1">
+        <f>+D28</f>
+        <v>19222.293399999999</v>
+      </c>
+      <c r="D39" s="1">
+        <f>+D30</f>
+        <v>25513.8871</v>
+      </c>
+      <c r="E39" s="1">
+        <v>0</v>
+      </c>
+      <c r="F39" s="1">
+        <f>-D28</f>
+        <v>-19222.293399999999</v>
+      </c>
+      <c r="G39" s="1">
+        <f>+D29</f>
+        <v>51375.286599999999</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B40" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B41" s="1">
+        <v>994802.49199999997</v>
+      </c>
+      <c r="C41" s="1">
+        <v>0</v>
+      </c>
+      <c r="D41" s="1">
+        <v>0</v>
+      </c>
+      <c r="E41" s="1">
+        <v>-994802.49199999997</v>
+      </c>
+      <c r="F41" s="1">
+        <v>0</v>
+      </c>
+      <c r="G41" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B42" s="1">
+        <v>0</v>
+      </c>
+      <c r="C42" s="1">
+        <v>9361.0023107912093</v>
+      </c>
+      <c r="D42" s="1">
+        <v>19222.0046215824</v>
+      </c>
+      <c r="E42" s="1">
+        <v>0</v>
+      </c>
+      <c r="F42" s="1">
+        <v>-9361.0023107912093</v>
+      </c>
+      <c r="G42" s="1">
+        <v>19222.0046215824</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B43" s="1">
+        <v>0</v>
+      </c>
+      <c r="C43" s="1">
+        <v>19222.0046215824</v>
+      </c>
+      <c r="D43" s="1">
+        <v>51372.767588837502</v>
+      </c>
+      <c r="E43" s="1">
+        <v>0</v>
+      </c>
+      <c r="F43" s="1">
+        <v>-19222.0046215824</v>
+      </c>
+      <c r="G43" s="1">
+        <v>25515.250897492198</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B44" s="1">
+        <v>-994802.49199999997</v>
+      </c>
+      <c r="C44" s="1">
+        <v>0</v>
+      </c>
+      <c r="D44" s="1">
+        <v>0</v>
+      </c>
+      <c r="E44" s="1">
+        <v>994802.49199999997</v>
+      </c>
+      <c r="F44" s="1">
+        <v>0</v>
+      </c>
+      <c r="G44" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B45" s="1">
+        <v>0</v>
+      </c>
+      <c r="C45" s="1">
+        <v>-9361.0023107912093</v>
+      </c>
+      <c r="D45" s="1">
+        <v>-19222.0046215824</v>
+      </c>
+      <c r="E45" s="1">
+        <v>0</v>
+      </c>
+      <c r="F45" s="1">
+        <v>9361.0023107912093</v>
+      </c>
+      <c r="G45" s="1">
+        <v>-19222.0046215824</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B46" s="1">
+        <v>0</v>
+      </c>
+      <c r="C46" s="1">
+        <v>19222.0046215824</v>
+      </c>
+      <c r="D46" s="1">
+        <v>25515.250897492198</v>
+      </c>
+      <c r="E46" s="1">
+        <v>0</v>
+      </c>
+      <c r="F46" s="1">
+        <v>-19222.0046215824</v>
+      </c>
+      <c r="G46" s="1">
+        <v>51372.767588837502</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B56" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B40:G40"/>
+    <mergeCell ref="B33:G33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>